<commit_message>
defaulted demo-cbm-hwp landfill off
</commit_message>
<xml_diff>
--- a/models/demo-cbm-hwp/demo-cbm-hwp.xlsx
+++ b/models/demo-cbm-hwp/demo-cbm-hwp.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shxie/projects/anse-models/demo-cbm-hwp/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shxie/projects/anse-public-releases/models/demo-cbm-hwp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D95CED6-6384-EF45-B4E8-5B2F1AAAE512}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE40CCD0-75A5-0A4C-9D45-419AF9931659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22960" yWindow="600" windowWidth="28240" windowHeight="26900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -854,9 +854,6 @@
     <t>CURVE_POINT</t>
   </si>
   <si>
-    <t>ON</t>
-  </si>
-  <si>
     <t>Landfilled Wood, Boreal Wet</t>
   </si>
   <si>
@@ -867,6 +864,9 @@
   </si>
   <si>
     <t>the rest should be all paper</t>
+  </si>
+  <si>
+    <t>OFF</t>
   </si>
 </sst>
 </file>
@@ -1781,7 +1781,7 @@
     <row r="24" spans="1:12" ht="16" customHeight="1">
       <c r="A24" s="5" t="str">
         <f>IF('Inputs - Landfill Module'!$C$3="OFF","","COMMENT")</f>
-        <v>COMMENT</v>
+        <v/>
       </c>
       <c r="B24" s="5" t="s">
         <v>23</v>
@@ -2095,7 +2095,7 @@
     <row r="48" spans="1:6" ht="16" customHeight="1">
       <c r="A48" s="5" t="str">
         <f>IF('Inputs - Landfill Module'!$C$3="OFF","","COMMENT")</f>
-        <v>COMMENT</v>
+        <v/>
       </c>
       <c r="B48" s="5" t="s">
         <v>32</v>
@@ -2118,7 +2118,7 @@
     <row r="49" spans="1:10" ht="16" customHeight="1">
       <c r="A49" s="5" t="str">
         <f>IF('Inputs - Landfill Module'!$C$3="OFF","","COMMENT")</f>
-        <v>COMMENT</v>
+        <v/>
       </c>
       <c r="B49" s="5" t="s">
         <v>32</v>
@@ -2638,7 +2638,7 @@
     <row r="86" spans="1:5" ht="16" customHeight="1">
       <c r="A86" s="5" t="str">
         <f>IF('Inputs - Landfill Module'!$C$3="OFF","","COMMENT")</f>
-        <v>COMMENT</v>
+        <v/>
       </c>
       <c r="B86" s="5" t="s">
         <v>47</v>
@@ -2728,7 +2728,7 @@
         <v>116</v>
       </c>
       <c r="C3" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:12" s="4" customFormat="1" ht="16" customHeight="1">
@@ -2770,7 +2770,7 @@
     <row r="7" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A7" s="5" t="str">
         <f>IF($C$3="ON","","COMMENT")</f>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>11</v>
@@ -2782,7 +2782,7 @@
     <row r="8" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A8" s="5" t="str">
         <f t="shared" ref="A8:A22" si="0">IF($C$3="ON","","COMMENT")</f>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>11</v>
@@ -2794,13 +2794,13 @@
     <row r="9" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A9" s="5" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="10" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A10" s="5" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>11</v>
@@ -2812,7 +2812,7 @@
     <row r="11" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A11" s="5" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>11</v>
@@ -2824,19 +2824,19 @@
     <row r="12" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A12" s="5" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="13" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A13" s="5" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>11</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E13" s="5" t="str">
         <f>'Inputs - Curves'!C8</f>
@@ -2846,13 +2846,13 @@
     <row r="14" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A14" s="5" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>11</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E14" s="5" t="str">
         <f>'Inputs - Curves'!C9</f>
@@ -2862,13 +2862,13 @@
     <row r="15" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A15" s="5" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="16" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A16" s="5" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>11</v>
@@ -2880,13 +2880,13 @@
     <row r="17" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A17" s="5" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="18" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A18" s="5" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>11</v>
@@ -2898,7 +2898,7 @@
     <row r="19" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A19" s="5" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>11</v>
@@ -2910,7 +2910,7 @@
     <row r="20" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A20" s="5" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>11</v>
@@ -2922,13 +2922,13 @@
     <row r="21" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A21" s="5" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="22" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A22" s="5" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>11</v>
@@ -2977,7 +2977,7 @@
     <row r="26" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A26" s="5" t="str">
         <f t="shared" ref="A26" si="1">IF($C$3="ON","","COMMENT")</f>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>23</v>
@@ -2989,7 +2989,7 @@
     <row r="27" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A27" s="5" t="str">
         <f t="shared" ref="A27:A34" si="2">IF($C$3="ON","","COMMENT")</f>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>23</v>
@@ -3001,7 +3001,7 @@
     <row r="28" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A28" s="5" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>23</v>
@@ -3013,7 +3013,7 @@
     <row r="29" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A29" s="5" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>23</v>
@@ -3025,7 +3025,7 @@
     <row r="30" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A30" s="5" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>23</v>
@@ -3037,7 +3037,7 @@
     <row r="31" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A31" s="5" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>23</v>
@@ -3049,7 +3049,7 @@
     <row r="32" spans="1:12" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A32" s="5" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>23</v>
@@ -3061,7 +3061,7 @@
     <row r="33" spans="1:7" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A33" s="5" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>23</v>
@@ -3073,7 +3073,7 @@
     <row r="34" spans="1:7" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A34" s="5" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>23</v>
@@ -3116,7 +3116,7 @@
     <row r="40" spans="1:7" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A40" s="5" t="str">
         <f t="shared" ref="A40:A75" si="3">IF($C$3="ON","","COMMENT")</f>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>32</v>
@@ -3139,7 +3139,7 @@
     <row r="41" spans="1:7" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A41" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>32</v>
@@ -3162,7 +3162,7 @@
     <row r="42" spans="1:7" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A42" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B42" s="5" t="s">
         <v>32</v>
@@ -3185,13 +3185,13 @@
     <row r="43" spans="1:7" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A43" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="44" spans="1:7" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A44" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B44" s="5" t="s">
         <v>32</v>
@@ -3214,7 +3214,7 @@
     <row r="45" spans="1:7" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A45" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>32</v>
@@ -3237,7 +3237,7 @@
     <row r="46" spans="1:7" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A46" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B46" s="5" t="s">
         <v>32</v>
@@ -3260,13 +3260,13 @@
     <row r="47" spans="1:7" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A47" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="48" spans="1:7" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A48" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>32</v>
@@ -3289,7 +3289,7 @@
     <row r="49" spans="1:6" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A49" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B49" s="5" t="s">
         <v>32</v>
@@ -3312,7 +3312,7 @@
     <row r="50" spans="1:6" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A50" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>32</v>
@@ -3335,13 +3335,13 @@
     <row r="51" spans="1:6" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A51" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="52" spans="1:6" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A52" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>32</v>
@@ -3364,7 +3364,7 @@
     <row r="53" spans="1:6" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A53" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>32</v>
@@ -3387,7 +3387,7 @@
     <row r="54" spans="1:6" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A54" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>32</v>
@@ -3410,7 +3410,7 @@
     <row r="55" spans="1:6" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A55" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>32</v>
@@ -3433,13 +3433,13 @@
     <row r="56" spans="1:6" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A56" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="57" spans="1:6" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A57" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>32</v>
@@ -3462,7 +3462,7 @@
     <row r="58" spans="1:6" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A58" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B58" s="5" t="s">
         <v>32</v>
@@ -3485,7 +3485,7 @@
     <row r="59" spans="1:6" s="5" customFormat="1" ht="16" customHeight="1">
       <c r="A59" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>32</v>
@@ -3508,7 +3508,7 @@
     <row r="60" spans="1:6">
       <c r="A60" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>32</v>
@@ -3531,14 +3531,14 @@
     <row r="61" spans="1:6">
       <c r="A61" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B61" s="5"/>
     </row>
     <row r="62" spans="1:6">
       <c r="A62" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>32</v>
@@ -3561,7 +3561,7 @@
     <row r="63" spans="1:6">
       <c r="A63" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>32</v>
@@ -3584,7 +3584,7 @@
     <row r="64" spans="1:6">
       <c r="A64" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B64" s="5" t="s">
         <v>32</v>
@@ -3607,13 +3607,13 @@
     <row r="65" spans="1:10">
       <c r="A65" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B66" s="5" t="s">
         <v>32</v>
@@ -3636,7 +3636,7 @@
     <row r="67" spans="1:10">
       <c r="A67" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>32</v>
@@ -3659,7 +3659,7 @@
     <row r="68" spans="1:10">
       <c r="A68" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>32</v>
@@ -3682,14 +3682,14 @@
     <row r="69" spans="1:10">
       <c r="A69" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B69" s="5"/>
     </row>
     <row r="70" spans="1:10">
       <c r="A70" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B70" s="5" t="s">
         <v>32</v>
@@ -3712,7 +3712,7 @@
     <row r="71" spans="1:10">
       <c r="A71" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>32</v>
@@ -3735,7 +3735,7 @@
     <row r="72" spans="1:10">
       <c r="A72" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>32</v>
@@ -3758,14 +3758,14 @@
     <row r="73" spans="1:10">
       <c r="A73" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B73" s="5"/>
     </row>
     <row r="74" spans="1:10">
       <c r="A74" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B74" s="5" t="s">
         <v>32</v>
@@ -3788,7 +3788,7 @@
     <row r="75" spans="1:10">
       <c r="A75" s="5" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>32</v>
@@ -3866,7 +3866,7 @@
     <row r="81" spans="1:10">
       <c r="A81" s="5" t="str">
         <f t="shared" ref="A81:A112" si="11">IF($C$3="ON","","COMMENT")</f>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B81" s="5" t="s">
         <v>47</v>
@@ -3886,7 +3886,7 @@
     <row r="82" spans="1:10">
       <c r="A82" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B82" s="5" t="s">
         <v>47</v>
@@ -3906,14 +3906,14 @@
     <row r="83" spans="1:10">
       <c r="A83" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B83" s="5"/>
     </row>
     <row r="84" spans="1:10">
       <c r="A84" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B84" s="5" t="s">
         <v>47</v>
@@ -3937,7 +3937,7 @@
     <row r="85" spans="1:10">
       <c r="A85" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B85" s="5" t="s">
         <v>47</v>
@@ -3961,14 +3961,14 @@
     <row r="86" spans="1:10">
       <c r="A86" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B86" s="5"/>
     </row>
     <row r="87" spans="1:10">
       <c r="A87" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B87" s="5" t="s">
         <v>47</v>
@@ -3985,13 +3985,13 @@
         <v>0.5</v>
       </c>
       <c r="J87" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="88" spans="1:10">
       <c r="A88" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B88" s="5" t="s">
         <v>47</v>
@@ -4011,14 +4011,14 @@
     <row r="89" spans="1:10">
       <c r="A89" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B89" s="5"/>
     </row>
     <row r="90" spans="1:10">
       <c r="A90" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B90" s="5" t="s">
         <v>47</v>
@@ -4042,7 +4042,7 @@
     <row r="91" spans="1:10">
       <c r="A91" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B91" s="5" t="s">
         <v>47</v>
@@ -4102,20 +4102,20 @@
         <v>1</v>
       </c>
       <c r="J94" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="95" spans="1:10">
       <c r="A95" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B95" s="5"/>
     </row>
     <row r="96" spans="1:10">
       <c r="A96" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B96" s="5" t="s">
         <v>47</v>
@@ -4135,7 +4135,7 @@
     <row r="97" spans="1:5">
       <c r="A97" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B97" s="5" t="s">
         <v>47</v>
@@ -4155,14 +4155,14 @@
     <row r="98" spans="1:5">
       <c r="A98" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B98" s="5"/>
     </row>
     <row r="99" spans="1:5">
       <c r="A99" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B99" s="5" t="s">
         <v>47</v>
@@ -4182,7 +4182,7 @@
     <row r="100" spans="1:5">
       <c r="A100" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B100" s="5" t="s">
         <v>47</v>
@@ -4202,7 +4202,7 @@
     <row r="101" spans="1:5">
       <c r="A101" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B101" s="5" t="s">
         <v>47</v>
@@ -4222,14 +4222,14 @@
     <row r="102" spans="1:5">
       <c r="A102" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B102" s="5"/>
     </row>
     <row r="103" spans="1:5">
       <c r="A103" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B103" s="5" t="s">
         <v>47</v>
@@ -4249,7 +4249,7 @@
     <row r="104" spans="1:5">
       <c r="A104" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B104" s="5" t="s">
         <v>47</v>
@@ -4269,13 +4269,13 @@
     <row r="105" spans="1:5">
       <c r="A105" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="106" spans="1:5">
       <c r="A106" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B106" s="5" t="s">
         <v>47</v>
@@ -4295,7 +4295,7 @@
     <row r="107" spans="1:5">
       <c r="A107" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B107" s="5" t="s">
         <v>47</v>
@@ -4315,13 +4315,13 @@
     <row r="108" spans="1:5">
       <c r="A108" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="109" spans="1:5">
       <c r="A109" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B109" s="5" t="s">
         <v>47</v>
@@ -4341,7 +4341,7 @@
     <row r="110" spans="1:5">
       <c r="A110" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B110" s="5" t="s">
         <v>47</v>
@@ -4361,13 +4361,13 @@
     <row r="111" spans="1:5">
       <c r="A111" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="112" spans="1:5">
       <c r="A112" s="5" t="str">
         <f t="shared" si="11"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B112" s="5" t="s">
         <v>47</v>
@@ -4409,7 +4409,7 @@
       <c r="B120" s="5"/>
     </row>
   </sheetData>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C3" xr:uid="{39B9DEFA-7EEB-5749-872D-4B58745AD69B}">
       <formula1>"ON, OFF"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
uncomment cbm-hwp model inputs
</commit_message>
<xml_diff>
--- a/models/demo-cbm-hwp/demo-cbm-hwp.xlsx
+++ b/models/demo-cbm-hwp/demo-cbm-hwp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shxie/projects/anse-models/demo-cbm-hwp/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shxie/projects/anse-public-releases/models/demo-cbm-hwp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5258F10-B1AC-9E49-9994-CC9F4D4BA33F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3B946D7-90E6-C943-BA8A-31D537D69FE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="32680" windowHeight="21320" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="32680" windowHeight="21320" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs - Flow Network" sheetId="1" r:id="rId1"/>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="142">
   <si>
     <t>Keyword: POOL</t>
   </si>
@@ -513,7 +513,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -548,12 +548,6 @@
       <color theme="1"/>
       <name val="HelveticaNeue"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -4017,7 +4011,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K37"/>
+  <dimension ref="B1:K37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.5703125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="19.5703125" customWidth="1"/>
@@ -4031,7 +4025,7 @@
     <col min="9" max="11" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="6" customFormat="1">
+    <row r="1" spans="2:11" s="6" customFormat="1">
       <c r="B1" s="7" t="s">
         <v>88</v>
       </c>
@@ -4063,10 +4057,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
-      <c r="A3" t="s">
-        <v>61</v>
-      </c>
+    <row r="3" spans="2:11">
       <c r="B3" t="s">
         <v>97</v>
       </c>
@@ -4082,10 +4073,7 @@
         <v>1990</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
-      <c r="A4" t="s">
-        <v>61</v>
-      </c>
+    <row r="4" spans="2:11">
       <c r="B4" t="s">
         <v>97</v>
       </c>
@@ -4101,10 +4089,7 @@
         <v>1991</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
-      <c r="A5" t="s">
-        <v>61</v>
-      </c>
+    <row r="5" spans="2:11">
       <c r="B5" t="s">
         <v>97</v>
       </c>
@@ -4120,10 +4105,7 @@
         <v>1992</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
-      <c r="A6" t="s">
-        <v>61</v>
-      </c>
+    <row r="6" spans="2:11">
       <c r="B6" t="s">
         <v>97</v>
       </c>
@@ -4139,10 +4121,7 @@
         <v>1993</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
-      <c r="A7" t="s">
-        <v>61</v>
-      </c>
+    <row r="7" spans="2:11">
       <c r="B7" t="s">
         <v>97</v>
       </c>
@@ -4158,10 +4137,7 @@
         <v>1994</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
-      <c r="A8" t="s">
-        <v>61</v>
-      </c>
+    <row r="8" spans="2:11">
       <c r="B8" t="s">
         <v>97</v>
       </c>
@@ -4177,10 +4153,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
-      <c r="A9" t="s">
-        <v>61</v>
-      </c>
+    <row r="9" spans="2:11">
       <c r="B9" t="s">
         <v>97</v>
       </c>
@@ -4196,10 +4169,7 @@
         <v>1996</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
-      <c r="A10" t="s">
-        <v>61</v>
-      </c>
+    <row r="10" spans="2:11">
       <c r="B10" t="s">
         <v>97</v>
       </c>
@@ -4215,10 +4185,7 @@
         <v>1997</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
-      <c r="A11" t="s">
-        <v>61</v>
-      </c>
+    <row r="11" spans="2:11">
       <c r="B11" t="s">
         <v>97</v>
       </c>
@@ -4234,10 +4201,7 @@
         <v>1998</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
-      <c r="A12" t="s">
-        <v>61</v>
-      </c>
+    <row r="12" spans="2:11">
       <c r="B12" t="s">
         <v>97</v>
       </c>
@@ -4253,10 +4217,7 @@
         <v>1999</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
-      <c r="A13" t="s">
-        <v>61</v>
-      </c>
+    <row r="13" spans="2:11">
       <c r="B13" t="s">
         <v>97</v>
       </c>
@@ -4272,10 +4233,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
-      <c r="A14" t="s">
-        <v>61</v>
-      </c>
+    <row r="14" spans="2:11">
       <c r="B14" t="s">
         <v>97</v>
       </c>
@@ -4291,10 +4249,7 @@
         <v>2001</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
-      <c r="A15" t="s">
-        <v>61</v>
-      </c>
+    <row r="15" spans="2:11">
       <c r="B15" t="s">
         <v>97</v>
       </c>
@@ -4310,10 +4265,7 @@
         <v>2002</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
-      <c r="A16" t="s">
-        <v>61</v>
-      </c>
+    <row r="16" spans="2:11">
       <c r="B16" t="s">
         <v>97</v>
       </c>
@@ -4329,10 +4281,7 @@
         <v>2003</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
-      <c r="A17" t="s">
-        <v>61</v>
-      </c>
+    <row r="17" spans="2:7">
       <c r="B17" t="s">
         <v>97</v>
       </c>
@@ -4348,10 +4297,7 @@
         <v>2004</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
-      <c r="A18" t="s">
-        <v>61</v>
-      </c>
+    <row r="18" spans="2:7">
       <c r="B18" t="s">
         <v>97</v>
       </c>
@@ -4367,10 +4313,7 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
-      <c r="A19" t="s">
-        <v>61</v>
-      </c>
+    <row r="19" spans="2:7">
       <c r="B19" t="s">
         <v>97</v>
       </c>
@@ -4386,10 +4329,7 @@
         <v>2006</v>
       </c>
     </row>
-    <row r="20" spans="1:7">
-      <c r="A20" t="s">
-        <v>61</v>
-      </c>
+    <row r="20" spans="2:7">
       <c r="B20" t="s">
         <v>97</v>
       </c>
@@ -4405,10 +4345,7 @@
         <v>2007</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
-      <c r="A21" t="s">
-        <v>61</v>
-      </c>
+    <row r="21" spans="2:7">
       <c r="B21" t="s">
         <v>97</v>
       </c>
@@ -4424,10 +4361,7 @@
         <v>2008</v>
       </c>
     </row>
-    <row r="22" spans="1:7">
-      <c r="A22" t="s">
-        <v>61</v>
-      </c>
+    <row r="22" spans="2:7">
       <c r="B22" t="s">
         <v>97</v>
       </c>
@@ -4443,10 +4377,7 @@
         <v>2009</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
-      <c r="A23" t="s">
-        <v>61</v>
-      </c>
+    <row r="23" spans="2:7">
       <c r="B23" t="s">
         <v>97</v>
       </c>
@@ -4462,10 +4393,7 @@
         <v>2010</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
-      <c r="A24" t="s">
-        <v>61</v>
-      </c>
+    <row r="24" spans="2:7">
       <c r="B24" t="s">
         <v>97</v>
       </c>
@@ -4481,10 +4409,7 @@
         <v>2011</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
-      <c r="A25" t="s">
-        <v>61</v>
-      </c>
+    <row r="25" spans="2:7">
       <c r="B25" t="s">
         <v>97</v>
       </c>
@@ -4500,10 +4425,7 @@
         <v>2012</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
-      <c r="A26" t="s">
-        <v>61</v>
-      </c>
+    <row r="26" spans="2:7">
       <c r="B26" t="s">
         <v>97</v>
       </c>
@@ -4519,10 +4441,7 @@
         <v>2013</v>
       </c>
     </row>
-    <row r="27" spans="1:7">
-      <c r="A27" t="s">
-        <v>61</v>
-      </c>
+    <row r="27" spans="2:7">
       <c r="B27" t="s">
         <v>97</v>
       </c>
@@ -4538,10 +4457,7 @@
         <v>2014</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
-      <c r="A28" t="s">
-        <v>61</v>
-      </c>
+    <row r="28" spans="2:7">
       <c r="B28" t="s">
         <v>97</v>
       </c>
@@ -4557,10 +4473,7 @@
         <v>2015</v>
       </c>
     </row>
-    <row r="29" spans="1:7">
-      <c r="A29" t="s">
-        <v>61</v>
-      </c>
+    <row r="29" spans="2:7">
       <c r="B29" t="s">
         <v>97</v>
       </c>
@@ -4576,10 +4489,7 @@
         <v>2016</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
-      <c r="A30" t="s">
-        <v>61</v>
-      </c>
+    <row r="30" spans="2:7">
       <c r="B30" t="s">
         <v>97</v>
       </c>
@@ -4595,10 +4505,7 @@
         <v>2017</v>
       </c>
     </row>
-    <row r="31" spans="1:7">
-      <c r="A31" t="s">
-        <v>61</v>
-      </c>
+    <row r="31" spans="2:7">
       <c r="B31" t="s">
         <v>97</v>
       </c>
@@ -4614,10 +4521,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="32" spans="1:7">
-      <c r="A32" t="s">
-        <v>61</v>
-      </c>
+    <row r="32" spans="2:7">
       <c r="B32" t="s">
         <v>97</v>
       </c>
@@ -4633,10 +4537,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="33" spans="1:7">
-      <c r="A33" t="s">
-        <v>61</v>
-      </c>
+    <row r="33" spans="2:7">
       <c r="B33" t="s">
         <v>97</v>
       </c>
@@ -4652,10 +4553,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="34" spans="1:7">
-      <c r="A34" t="s">
-        <v>61</v>
-      </c>
+    <row r="34" spans="2:7">
       <c r="B34" t="s">
         <v>97</v>
       </c>
@@ -4671,10 +4569,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
-      <c r="A35" t="s">
-        <v>61</v>
-      </c>
+    <row r="35" spans="2:7">
       <c r="B35" t="s">
         <v>97</v>
       </c>
@@ -4690,10 +4585,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
-      <c r="A36" t="s">
-        <v>61</v>
-      </c>
+    <row r="36" spans="2:7">
       <c r="B36" t="s">
         <v>97</v>
       </c>
@@ -4709,10 +4601,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="37" spans="1:7">
-      <c r="A37" t="s">
-        <v>61</v>
-      </c>
+    <row r="37" spans="2:7">
       <c r="B37" t="s">
         <v>97</v>
       </c>

</xml_diff>